<commit_message>
Add student name section to START HERE
</commit_message>
<xml_diff>
--- a/Patient_Access_Bottleneck_Intelligence_System.xlsx
+++ b/Patient_Access_Bottleneck_Intelligence_System.xlsx
@@ -29,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -112,6 +112,12 @@
       <color rgb="001A1A1A"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -187,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -264,6 +270,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -759,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -783,225 +794,212 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Created by Kori Pickle · BSHA Candidate, University of Phoenix · Degree in progress · No formal healthcare employment</t>
+      <c r="A3" s="34" t="inlineStr">
+        <is>
+          <t>Student: Kori Pickle  ·  BSHA Candidate, University of Phoenix  ·  Degree in progress  ·  No formal healthcare employment</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>STUDENT</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Kori Pickle</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Bachelor of Science in Healthcare Administration (in progress), University of Phoenix</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Undergraduate student · No formal healthcare employment experience</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1"/>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>PROJECT PURPOSE</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="B10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Trace where a simulated patient-access workflow first loses control, show the downstream effect, and practice the controls needed to restore the case.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Simulated problem</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>An inaccurate demographic element entered during registration creates an eligibility mismatch. That mismatch delays authorization readiness, financial clearance, patient communication, and verified closure.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>What this artifact demonstrates</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Workflow mapping, case organization, prioritization, ownership assignment, follow-up logic, escalation rules, accuracy controls, patient-communication status tracking, and formula-driven dashboard interpretation.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>What this artifact does not claim</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>No formal healthcare employment, live patient registration, payer-portal work, EHR access, measured operational results, or professional compliance authority.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Integrity statement</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>All names, identifiers, dates, payers, records, and outcomes in this workbook are synthetic. No real patient, payer, or employer data is used.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+    <row r="16" ht="28" customHeight="1"/>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>HOW TO USE THE WORKBOOK</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n"/>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Review WORKFLOW MAP to understand the simulated failure path and the control that should have stopped it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Use CASE CONTROL to examine ownership, priority, next action, follow-up, escalation, communication, and closure for each simulated case.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Use ACCURACY CONTROLS to verify what must be checked before a case moves downstream or is closed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Use RISK MATRIX to see which failure types carry higher downstream impact and how they are prioritized.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Use DASHBOARD to summarize open workload, bottleneck stage, escalations, overdue follow-ups, and closure status.</t>
-        </is>
-      </c>
+      <c r="B17" s="5" t="n"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Use GLOSSARY for plain-language definitions of the terms used in the workbook.</t>
+          <t>Review WORKFLOW MAP to understand the simulated failure path and the control that should have stopped it.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Use CASE CONTROL to examine ownership, priority, next action, follow-up, escalation, communication, and closure for each simulated case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Use ACCURACY CONTROLS to verify what must be checked before a case moves downstream or is closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Use RISK MATRIX to see which failure types carry higher downstream impact and how they are prioritized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Use DASHBOARD to summarize open workload, bottleneck stage, escalations, overdue follow-ups, and closure status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Use GLOSSARY for plain-language definitions of the terms used in the workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Use EVIDENCE GUIDE for résumé wording and interview talking points that stay within honest student boundaries.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>COMPLETION STANDARD</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Workflow path identifies the earliest loss of control.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Every simulated case has an owner, next action, follow-up date, and status.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>Escalation logic is visible and applied consistently.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>Patient communication status is tracked without including PHI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>Closure requires documented evidence and a final accuracy check.</t>
-        </is>
-      </c>
+      <c r="B26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -1011,7 +1009,7 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Dashboard metrics reconcile to the case-control table.</t>
+          <t>Workflow path identifies the earliest loss of control.</t>
         </is>
       </c>
     </row>
@@ -1022,6 +1020,66 @@
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Every simulated case has an owner, next action, follow-up date, and status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Escalation logic is visible and applied consistently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Patient communication status is tracked without including PHI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Closure requires documented evidence and a final accuracy check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard metrics reconcile to the case-control table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Risk rating is assigned and visible for each open case.</t>
         </is>
@@ -1075,6 +1133,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -1494,6 +1553,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -2768,6 +2828,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -3081,6 +3142,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -3352,14 +3414,15 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t>WORKLOAD SUMMARY</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="36" t="inlineStr">
         <is>
           <t>OPEN CASES BY STAGE</t>
         </is>
@@ -3548,6 +3611,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -3720,6 +3784,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -3875,7 +3940,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>RESUME BULLET (HONEST)</t>
         </is>
@@ -3892,7 +3957,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="36" t="inlineStr">
         <is>
           <t>60-SECOND INTERVIEW EXPLANATION</t>
         </is>
@@ -3909,7 +3974,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+      <c r="A18" s="36" t="inlineStr">
         <is>
           <t>PORTFOLIO DISCLAIMER</t>
         </is>

</xml_diff>

<commit_message>
Finalize PABIS workbook: 50 formulas, 3 dropdowns and closure controls
</commit_message>
<xml_diff>
--- a/Patient_Access_Bottleneck_Intelligence_System.xlsx
+++ b/Patient_Access_Bottleneck_Intelligence_System.xlsx
@@ -2488,12 +2488,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF8200"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.97265625" customWidth="1"/>
@@ -2625,6 +2625,11 @@
       <c r="T4" s="8" t="s">
         <v>125</v>
       </c>
+      <c r="U4" s="8" t="inlineStr">
+        <is>
+          <t>MODELED CLOSURE CONTROL</t>
+        </is>
+      </c>
     </row>
     <row r="5" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
@@ -2687,6 +2692,10 @@
       <c r="T5" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="U5" s="9">
+        <f>IF(P5&lt;&gt;"Closed","Not applicable",IF(OR(Q5="",R5="",S5&lt;&gt;"Pass",O5=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="6" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
@@ -2749,6 +2758,10 @@
       <c r="T6" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="U6" s="10">
+        <f>IF(P6&lt;&gt;"Closed","Not applicable",IF(OR(Q6="",R6="",S6&lt;&gt;"Pass",O6=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="7" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
@@ -2811,6 +2824,10 @@
       <c r="T7" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="U7" s="9">
+        <f>IF(P7&lt;&gt;"Closed","Not applicable",IF(OR(Q7="",R7="",S7&lt;&gt;"Pass",O7=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="8" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="10" t="s">
@@ -2873,6 +2890,10 @@
       <c r="T8" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="U8" s="10">
+        <f>IF(P8&lt;&gt;"Closed","Not applicable",IF(OR(Q8="",R8="",S8&lt;&gt;"Pass",O8=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="9" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
@@ -2935,6 +2956,10 @@
       <c r="T9" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="U9" s="9">
+        <f>IF(P9&lt;&gt;"Closed","Not applicable",IF(OR(Q9="",R9="",S9&lt;&gt;"Pass",O9=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="10" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
@@ -2999,6 +3024,10 @@
       <c r="T10" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="U10" s="10">
+        <f>IF(P10&lt;&gt;"Closed","Not applicable",IF(OR(Q10="",R10="",S10&lt;&gt;"Pass",O10=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="11" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
@@ -3063,6 +3092,10 @@
       <c r="T11" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="U11" s="9">
+        <f>IF(P11&lt;&gt;"Closed","Not applicable",IF(OR(Q11="",R11="",S11&lt;&gt;"Pass",O11=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="12" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
@@ -3125,6 +3158,10 @@
       <c r="T12" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="U12" s="10">
+        <f>IF(P12&lt;&gt;"Closed","Not applicable",IF(OR(Q12="",R12="",S12&lt;&gt;"Pass",O12=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="13" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
@@ -3187,6 +3224,10 @@
       <c r="T13" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="U13" s="9">
+        <f>IF(P13&lt;&gt;"Closed","Not applicable",IF(OR(Q13="",R13="",S13&lt;&gt;"Pass",O13=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="14" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
@@ -3249,6 +3290,10 @@
       <c r="T14" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="U14" s="10">
+        <f>IF(P14&lt;&gt;"Closed","Not applicable",IF(OR(Q14="",R14="",S14&lt;&gt;"Pass",O14=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="15" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
@@ -3311,6 +3356,10 @@
       <c r="T15" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="U15" s="9">
+        <f>IF(P15&lt;&gt;"Closed","Not applicable",IF(OR(Q15="",R15="",S15&lt;&gt;"Pass",O15=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
+      </c>
     </row>
     <row r="16" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
@@ -3374,6 +3423,10 @@
       </c>
       <c r="T16" s="10" t="s">
         <v>139</v>
+      </c>
+      <c r="U16" s="10">
+        <f>IF(P16&lt;&gt;"Closed","Not applicable",IF(OR(Q16="",R16="",S16&lt;&gt;"Pass",O16=""),"BLOCKED — review closure","Ready — modeled closure only"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3401,6 +3454,17 @@
       <formula>$P5="In Progress"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation type="list" sqref="H5:H16">
+      <formula1>"Low,Medium,High,Urgent"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="P5:P16">
+      <formula1>"Open,In Progress,Closed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="S5:S16">
+      <formula1>"Pending,Pass,Fail"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
@@ -3824,7 +3888,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF8200"/>
     <pageSetUpPr fitToPage="1"/>
@@ -3985,6 +4049,17 @@
       <c r="E11" s="20">
         <f>COUNTIFS('CASE CONTROL'!C5:C16,D11,'CASE CONTROL'!P5:P16,"&lt;&gt;Closed")</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Blocked modeled closures</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>COUNTIF('CASE CONTROL'!U5:U16,"BLOCKED*")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>